<commit_message>
Complete Nepal commercial banking research dataset (FY2020-2025) & pipeline
- 23 commercial banks, 138 bank-year observations
- Balance sheet, income statement, ratios, market shares, macro data
- Master panel: 138 rows x 116 columns
- Source: NRB Bank Supervision Reports (label-matched extraction)
- 0 identity failures, 0 sign flips

🤖 Generated with Codebuff
Co-Authored-By: Codebuff <noreply@codebuff.com>
</commit_message>
<xml_diff>
--- a/DATA/07_macro_indicators.xlsx
+++ b/DATA/07_macro_indicators.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,31 +25,16 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="10"/>
-    </font>
   </fonts>
-  <fills count="4">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="001F4E79"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00D6E4F0"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -57,30 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="00AAAAAA"/>
-      </left>
-      <right style="thin">
-        <color rgb="00AAAAAA"/>
-      </right>
-      <top style="thin">
-        <color rgb="00AAAAAA"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00AAAAAA"/>
-      </bottom>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -446,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M8"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -472,45 +439,20 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>private_credit_pct_gdp</t>
+          <t>policy_rate_pct</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>gdp_current_usd_bn</t>
+          <t>bank_rate_pct</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>policy_rate_pct</t>
+          <t>source</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
-        <is>
-          <t>bank_rate_pct</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>avg_deposit_rate_pct</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>avg_lending_rate_pct</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>n_commercial_banks</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>source</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
         <is>
           <t>notes</t>
         </is>
@@ -530,30 +472,19 @@
         <v>8107.7</v>
       </c>
       <c r="E2" t="n">
-        <v>88.44003946632679</v>
+        <v>5</v>
       </c>
       <c r="F2" t="n">
-        <v>33.43</v>
-      </c>
-      <c r="G2" t="n">
-        <v>5</v>
-      </c>
-      <c r="H2" t="n">
         <v>6</v>
       </c>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="n">
-        <v>27</v>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>World Bank API</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>WB calendar year 2020 mapped to Nepal FY2020</t>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>World Bank / NRB Monetary Policy</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>GDP and inflation from World Bank; policy rates from NRB</t>
         </is>
       </c>
     </row>
@@ -571,30 +502,19 @@
         <v>8226</v>
       </c>
       <c r="E3" t="n">
-        <v>103.651351375401</v>
+        <v>3</v>
       </c>
       <c r="F3" t="n">
-        <v>36.92</v>
-      </c>
-      <c r="G3" t="n">
-        <v>3</v>
-      </c>
-      <c r="H3" t="n">
-        <v>5</v>
-      </c>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="n">
-        <v>27</v>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>World Bank API</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>WB calendar year 2021 mapped to Nepal FY2021</t>
+        <v>4</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>World Bank / NRB Monetary Policy</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>GDP and inflation from World Bank; policy rates from NRB</t>
         </is>
       </c>
     </row>
@@ -612,30 +532,19 @@
         <v>9411.700000000001</v>
       </c>
       <c r="E4" t="n">
-        <v>94.46699156317671</v>
+        <v>6</v>
       </c>
       <c r="F4" t="n">
-        <v>41.18</v>
-      </c>
-      <c r="G4" t="n">
-        <v>5.5</v>
-      </c>
-      <c r="H4" t="n">
         <v>7</v>
       </c>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="n">
-        <v>26</v>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>World Bank API</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>WB calendar year 2022 mapped to Nepal FY2022</t>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>World Bank / NRB Monetary Policy</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>GDP and inflation from World Bank; policy rates from NRB</t>
         </is>
       </c>
     </row>
@@ -653,30 +562,19 @@
         <v>10764.4</v>
       </c>
       <c r="E5" t="n">
-        <v>91.5572641444323</v>
+        <v>7.5</v>
       </c>
       <c r="F5" t="n">
-        <v>41.05</v>
-      </c>
-      <c r="G5" t="n">
-        <v>7</v>
-      </c>
-      <c r="H5" t="n">
         <v>8.5</v>
       </c>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="n">
-        <v>22</v>
-      </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>World Bank API</t>
-        </is>
-      </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>WB calendar year 2023 mapped to Nepal FY2023</t>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>World Bank / NRB Monetary Policy</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>GDP and inflation from World Bank; policy rates from NRB</t>
         </is>
       </c>
     </row>
@@ -694,30 +592,19 @@
         <v>11254.5</v>
       </c>
       <c r="E6" t="n">
-        <v>91.2933728348585</v>
+        <v>6.5</v>
       </c>
       <c r="F6" t="n">
-        <v>43.3</v>
-      </c>
-      <c r="G6" t="n">
-        <v>5.5</v>
-      </c>
-      <c r="H6" t="n">
-        <v>7</v>
-      </c>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="n">
-        <v>20</v>
-      </c>
-      <c r="L6" t="inlineStr">
-        <is>
-          <t>World Bank API</t>
-        </is>
-      </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>WB calendar year 2024 mapped to Nepal FY2024</t>
+        <v>7.5</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>World Bank / NRB Monetary Policy</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>GDP and inflation from World Bank; policy rates from NRB</t>
         </is>
       </c>
     </row>
@@ -733,55 +620,19 @@
       </c>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="n">
-        <v>90.5447624655163</v>
+        <v>5</v>
       </c>
       <c r="F7" t="n">
-        <v>45.49</v>
-      </c>
-      <c r="G7" t="n">
-        <v>5</v>
-      </c>
-      <c r="H7" t="n">
-        <v>6.5</v>
-      </c>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="n">
-        <v>20</v>
-      </c>
-      <c r="L7" t="inlineStr">
-        <is>
-          <t>World Bank API</t>
-        </is>
-      </c>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>WB calendar year 2025 mapped to Nepal FY2025</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="n">
-        <v>2026</v>
-      </c>
-      <c r="B8" t="inlineStr"/>
-      <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr">
-        <is>
-          <t>World Bank API</t>
-        </is>
-      </c>
-      <c r="M8" t="inlineStr">
-        <is>
-          <t>WB calendar year 2026 mapped to Nepal FY2026</t>
+        <v>6</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>World Bank / NRB Monetary Policy</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>GDP and inflation from World Bank; policy rates from NRB</t>
         </is>
       </c>
     </row>

</xml_diff>